<commit_message>
refactor: Update expedition data files and enhance font asset configurations
- Modified expedition_event.xlsx and expedition.xlsx files to reflect updated event and expedition configurations.
- Enhanced font asset SDF configuration by adding new glyph metrics and adjusting existing ones for improved text rendering.
- Updated ExpeditionMainUI prefab to change overflow mode, optimizing text display settings for better UI performance.
- Refactored gameplay logic in ExpeditionCombatSessionController and ExpeditionFlowController to ensure proper handling of marble snapshots, improving combat session integrity.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/expedition_event.xlsx
+++ b/Configs/GameConfig/Datas/expedition_event.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="28">
   <si>
     <t>##var</t>
   </si>
@@ -1379,8 +1379,8 @@
       <c r="D8" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="5">
-        <v>1</v>
+      <c r="E8" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>18</v>
@@ -1431,8 +1431,8 @@
       <c r="B10" s="21"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
-      <c r="E10" s="5">
-        <v>2</v>
+      <c r="E10" s="5" t="s">
+        <v>24</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>24</v>

</xml_diff>